<commit_message>
docs: record thesis journal setup session
</commit_message>
<xml_diff>
--- a/Timelog.xlsx
+++ b/Timelog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matae\OneDrive\Desktop\Coding-Projects\local-play-bootstrap-main\Thesis_ML\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BC8308F-F527-4DA4-AD5F-E5087BB0C9AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2A0EEC1-F79E-4586-862D-1174B28F316E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1545" yWindow="4725" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Time Log" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Thesis ML - Time Log</t>
   </si>
@@ -82,6 +82,9 @@
   </si>
   <si>
     <t>Building claude prompt to architect the model size test.</t>
+  </si>
+  <si>
+    <t>Adding a weekly journal log to my repo and filling it out. Working on cleaning up various things and commiting the working repo tree and pushing to github.</t>
   </si>
 </sst>
 </file>
@@ -235,17 +238,17 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -561,13 +564,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
     </row>
     <row r="2" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -575,14 +578,14 @@
       </c>
       <c r="B2" s="2">
         <f>ROUND(SUM(D5:D304),2)</f>
-        <v>10.75</v>
+        <v>12.25</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D2" s="3">
         <f>COUNT(D5:D304)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>3</v>
@@ -681,17 +684,17 @@
       <c r="A9" s="6">
         <v>46264</v>
       </c>
-      <c r="B9" s="22">
+      <c r="B9" s="20">
         <v>0.6875</v>
       </c>
-      <c r="C9" s="22">
+      <c r="C9" s="20">
         <v>0.72916666666666663</v>
       </c>
-      <c r="D9" s="20">
+      <c r="D9" s="18">
         <f t="shared" si="0"/>
         <v>0.99999999999999911</v>
       </c>
-      <c r="E9" s="21" t="s">
+      <c r="E9" s="19" t="s">
         <v>14</v>
       </c>
     </row>
@@ -714,14 +717,22 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="14"/>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="E11" s="17"/>
+      <c r="A11" s="6">
+        <v>46266</v>
+      </c>
+      <c r="B11" s="15">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="C11" s="15">
+        <v>0.47916666666666669</v>
+      </c>
+      <c r="D11" s="16">
+        <f t="shared" si="0"/>
+        <v>1.5</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="10"/>

</xml_diff>